<commit_message>
Empty deadline cells for Finalized claims with a Latest Date Worked
In all workbooks, Days Until Deadline, Days Until Corrected Claim
Deadline, Days Until Appeal Deadline and Filing Deadline show empty for
these claims. Filing Deadline keeps its date inside a formula, so the
deadlines come back automatically if the status or Latest Date Worked
changes. These cells take the Finalized row colour, and the Read Me
deadline counts leave the claims out.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgCgUMEP34hb7McfZTNVaf
</commit_message>
<xml_diff>
--- a/SPC26S1 - 01 January v2.xlsx
+++ b/SPC26S1 - 01 January v2.xlsx
@@ -1928,7 +1928,7 @@
     <t>Every specialty sheet is sorted in four groups: Rejected claims at the very top, then claims with an empty Latest Date Worked (column K), then the other open claims, and Finalized and PAID claims at the bottom (a Finalized or PAID claim with an empty Latest Date Worked stays in the empty Latest Date Worked group). Within each group, rows are ordered by how close the claim is to its primary payer's timely filing deadline. Days Until Deadline (column L) carries the count: five days or less left is shaded red, a negative number means the filing window has already closed, and a blank means no limit is on file for that payer.</t>
   </si>
   <si>
-    <t>Deadline order within each group, with the colour band each row gets (these counts update automatically):</t>
+    <t>Deadline order within each group, with the colour band each row gets (these counts update automatically; Finalized claims with a Latest Date Worked have their deadline cells left empty and are not counted):</t>
   </si>
   <si>
     <t>'SPC26S1 - 00 Master v2.xlsx' (same folder) holds every claim for 2026 S1. Its Claim Status and Notes columns are formulas that read this file, so anything you type in columns A and B here shows up there. Keep both files in the same folder, keep the file name unchanged, and save this file before opening the master.</t>
@@ -3700,14 +3700,15 @@
         <v>-148</v>
       </c>
       <c r="M2" s="14">
-        <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($C2="","",$C2+365-TODAY()))</f>
         <v>159</v>
       </c>
       <c r="N2" s="14">
-        <f ca="1">IF($C2="","",$C2+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($C2="","",$C2+90-TODAY()))</f>
         <v>-116</v>
       </c>
       <c r="O2" s="7">
+        <f>IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",DATE(2026,5,14))</f>
         <v>46156</v>
       </c>
       <c r="P2" s="6" t="s">
@@ -3811,14 +3812,15 @@
         <v>-79</v>
       </c>
       <c r="M3" s="14">
-        <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($C3="","",$C3+365-TODAY()))</f>
         <v>131</v>
       </c>
       <c r="N3" s="14">
-        <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($C3="","",$C3+365-TODAY()))</f>
         <v>131</v>
       </c>
       <c r="O3" s="7">
+        <f>IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",DATE(2026,7,22))</f>
         <v>46225</v>
       </c>
       <c r="P3" s="6" t="s">
@@ -3920,14 +3922,15 @@
         <v>104</v>
       </c>
       <c r="M4" s="14">
-        <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($C4="","",$C4+365-TODAY()))</f>
         <v>132</v>
       </c>
       <c r="N4" s="14">
-        <f ca="1">IF($C4="","",$C4+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($C4="","",$C4+120-TODAY()))</f>
         <v>-113</v>
       </c>
       <c r="O4" s="7">
+        <f>IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",DATE(2027,1,21))</f>
         <v>46408</v>
       </c>
       <c r="P4" s="6" t="s">
@@ -4029,14 +4032,15 @@
         <v>105</v>
       </c>
       <c r="M5" s="14">
-        <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($C5="","",$C5+365-TODAY()))</f>
         <v>190</v>
       </c>
       <c r="N5" s="14">
-        <f ca="1">IF($C5="","",$C5+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($C5="","",$C5+120-TODAY()))</f>
         <v>-55</v>
       </c>
       <c r="O5" s="7">
+        <f>IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",DATE(2027,1,22))</f>
         <v>46409</v>
       </c>
       <c r="P5" s="6" t="s">
@@ -4138,14 +4142,15 @@
         <v>111</v>
       </c>
       <c r="M6" s="14">
-        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($C6="","",$C6+365-TODAY()))</f>
         <v>133</v>
       </c>
       <c r="N6" s="14">
-        <f ca="1">IF($C6="","",$C6+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($C6="","",$C6+120-TODAY()))</f>
         <v>-112</v>
       </c>
       <c r="O6" s="7">
+        <f>IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",DATE(2027,1,28))</f>
         <v>46415</v>
       </c>
       <c r="P6" s="6" t="s">
@@ -4249,14 +4254,15 @@
         <v>-185</v>
       </c>
       <c r="M7" s="14">
-        <f ca="1">IF($F7="","",$F7+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($F7="","",$F7+90-TODAY()))</f>
         <v>-185</v>
       </c>
       <c r="N7" s="14">
-        <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($C7="","",$C7+365-TODAY()))</f>
         <v>124</v>
       </c>
       <c r="O7" s="7">
+        <f>IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",DATE(2026,4,7))</f>
         <v>46119</v>
       </c>
       <c r="P7" s="6" t="s">
@@ -4358,14 +4364,15 @@
         <v>-183</v>
       </c>
       <c r="M8" s="14">
-        <f ca="1">IF($C8="","",$C8+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($C8="","",$C8+180-TODAY()))</f>
         <v>17</v>
       </c>
       <c r="N8" s="14">
-        <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($C8="","",$C8+365-TODAY()))</f>
         <v>202</v>
       </c>
       <c r="O8" s="7">
+        <f>IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",DATE(2026,4,9))</f>
         <v>46121</v>
       </c>
       <c r="P8" s="6" t="s">
@@ -4469,14 +4476,15 @@
         <v>-186</v>
       </c>
       <c r="M9" s="14">
-        <f ca="1">IF($C9="","",$C9+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A9)="Finalized",$K9&lt;&gt;""),"",IF($C9="","",$C9+180-TODAY()))</f>
         <v>18</v>
       </c>
       <c r="N9" s="14">
-        <f ca="1">IF($C9="","",$C9+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A9)="Finalized",$K9&lt;&gt;""),"",IF($C9="","",$C9+365-TODAY()))</f>
         <v>203</v>
       </c>
       <c r="O9" s="7">
+        <f>IF(AND(TRIM($A9)="Finalized",$K9&lt;&gt;""),"",DATE(2026,4,6))</f>
         <v>46118</v>
       </c>
       <c r="P9" s="6" t="s">
@@ -4580,14 +4588,15 @@
         <v>-178</v>
       </c>
       <c r="M10" s="14">
-        <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A10)="Finalized",$K10&lt;&gt;""),"",IF($C10="","",$C10+365-TODAY()))</f>
         <v>194</v>
       </c>
       <c r="N10" s="14">
-        <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A10)="Finalized",$K10&lt;&gt;""),"",IF($C10="","",$C10+365-TODAY()))</f>
         <v>194</v>
       </c>
       <c r="O10" s="7">
+        <f>IF(AND(TRIM($A10)="Finalized",$K10&lt;&gt;""),"",DATE(2026,4,14))</f>
         <v>46126</v>
       </c>
       <c r="P10" s="6" t="s">
@@ -4691,14 +4700,15 @@
         <v>-171</v>
       </c>
       <c r="M11" s="14">
-        <f ca="1">IF($F11="","",$F11+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A11)="Finalized",$K11&lt;&gt;""),"",IF($F11="","",$F11+90-TODAY()))</f>
         <v>-171</v>
       </c>
       <c r="N11" s="14">
-        <f ca="1">IF($C11="","",$C11+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A11)="Finalized",$K11&lt;&gt;""),"",IF($C11="","",$C11+365-TODAY()))</f>
         <v>125</v>
       </c>
       <c r="O11" s="7">
+        <f>IF(AND(TRIM($A11)="Finalized",$K11&lt;&gt;""),"",DATE(2026,4,21))</f>
         <v>46133</v>
       </c>
       <c r="P11" s="6" t="s">
@@ -4802,14 +4812,15 @@
         <v>-170</v>
       </c>
       <c r="M12" s="14">
-        <f ca="1">IF($F12="","",$F12+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A12)="Finalized",$K12&lt;&gt;""),"",IF($F12="","",$F12+90-TODAY()))</f>
         <v>-170</v>
       </c>
       <c r="N12" s="14">
-        <f ca="1">IF($C12="","",$C12+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A12)="Finalized",$K12&lt;&gt;""),"",IF($C12="","",$C12+365-TODAY()))</f>
         <v>155</v>
       </c>
       <c r="O12" s="7">
+        <f>IF(AND(TRIM($A12)="Finalized",$K12&lt;&gt;""),"",DATE(2026,4,22))</f>
         <v>46134</v>
       </c>
       <c r="P12" s="6" t="s">
@@ -4915,14 +4926,15 @@
         <v>-165</v>
       </c>
       <c r="M13" s="14">
-        <f ca="1">IF($F13="","",$F13+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A13)="Finalized",$K13&lt;&gt;""),"",IF($F13="","",$F13+90-TODAY()))</f>
         <v>-165</v>
       </c>
       <c r="N13" s="14">
-        <f ca="1">IF($C13="","",$C13+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A13)="Finalized",$K13&lt;&gt;""),"",IF($C13="","",$C13+365-TODAY()))</f>
         <v>189</v>
       </c>
       <c r="O13" s="7">
+        <f>IF(AND(TRIM($A13)="Finalized",$K13&lt;&gt;""),"",DATE(2026,4,27))</f>
         <v>46139</v>
       </c>
       <c r="P13" s="6" t="s">
@@ -5026,14 +5038,15 @@
         <v>-165</v>
       </c>
       <c r="M14" s="14">
-        <f ca="1">IF($C14="","",$C14+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A14)="Finalized",$K14&lt;&gt;""),"",IF($C14="","",$C14+365-TODAY()))</f>
         <v>348</v>
       </c>
       <c r="N14" s="14">
-        <f ca="1">IF($C14="","",$C14+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A14)="Finalized",$K14&lt;&gt;""),"",IF($C14="","",$C14+365-TODAY()))</f>
         <v>348</v>
       </c>
       <c r="O14" s="7">
+        <f>IF(AND(TRIM($A14)="Finalized",$K14&lt;&gt;""),"",DATE(2026,4,27))</f>
         <v>46139</v>
       </c>
       <c r="P14" s="6" t="s">
@@ -5139,14 +5152,15 @@
         <v>-163</v>
       </c>
       <c r="M15" s="14">
-        <f ca="1">IF($F15="","",$F15+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A15)="Finalized",$K15&lt;&gt;""),"",IF($F15="","",$F15+90-TODAY()))</f>
         <v>-163</v>
       </c>
       <c r="N15" s="14">
-        <f ca="1">IF($C15="","",$C15+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A15)="Finalized",$K15&lt;&gt;""),"",IF($C15="","",$C15+365-TODAY()))</f>
         <v>127</v>
       </c>
       <c r="O15" s="7">
+        <f>IF(AND(TRIM($A15)="Finalized",$K15&lt;&gt;""),"",DATE(2026,4,29))</f>
         <v>46141</v>
       </c>
       <c r="P15" s="6" t="s">
@@ -5250,14 +5264,15 @@
         <v>-74</v>
       </c>
       <c r="M16" s="14">
-        <f ca="1">IF($F16="","",$F16+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A16)="Finalized",$K16&lt;&gt;""),"",IF($F16="","",$F16+365-TODAY()))</f>
         <v>111</v>
       </c>
       <c r="N16" s="14">
-        <f ca="1">IF($F16="","",$F16+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A16)="Finalized",$K16&lt;&gt;""),"",IF($F16="","",$F16+365-TODAY()))</f>
         <v>111</v>
       </c>
       <c r="O16" s="7">
+        <f>IF(AND(TRIM($A16)="Finalized",$K16&lt;&gt;""),"",DATE(2026,7,27))</f>
         <v>46230</v>
       </c>
       <c r="P16" s="6" t="s">
@@ -5361,14 +5376,15 @@
         <v>92</v>
       </c>
       <c r="M17" s="14">
-        <f ca="1">IF($C17="","",$C17+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A17)="Finalized",$K17&lt;&gt;""),"",IF($C17="","",$C17+365-TODAY()))</f>
         <v>132</v>
       </c>
       <c r="N17" s="14">
-        <f ca="1">IF($C17="","",$C17+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A17)="Finalized",$K17&lt;&gt;""),"",IF($C17="","",$C17+120-TODAY()))</f>
         <v>-113</v>
       </c>
       <c r="O17" s="7">
+        <f>IF(AND(TRIM($A17)="Finalized",$K17&lt;&gt;""),"",DATE(2027,1,9))</f>
         <v>46396</v>
       </c>
       <c r="P17" s="6" t="s">
@@ -5437,100 +5453,105 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AN17" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="L2:O1000">
+    <cfRule type="expression" dxfId="101" priority="1" stopIfTrue="1">
+      <formula>AND(TRIM($A2)="Finalized",$K2&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L2:L17">
-    <cfRule type="expression" dxfId="99" priority="1">
+    <cfRule type="expression" dxfId="99" priority="2">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="98" priority="2">
+    <cfRule type="expression" dxfId="98" priority="3">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="97" priority="3">
+    <cfRule type="expression" dxfId="97" priority="4">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="96" priority="4">
+    <cfRule type="expression" dxfId="96" priority="5">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="95" priority="5">
+    <cfRule type="expression" dxfId="95" priority="6">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M17">
-    <cfRule type="expression" dxfId="94" priority="6">
+    <cfRule type="expression" dxfId="94" priority="7">
       <formula>AND($M2&lt;&gt;"", $M2&gt;=0, $M2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="93" priority="7">
+    <cfRule type="expression" dxfId="93" priority="8">
       <formula>AND($M2&lt;&gt;"", $M2&gt;5, $M2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="92" priority="8">
+    <cfRule type="expression" dxfId="92" priority="9">
       <formula>AND($M2&lt;&gt;"", $M2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="91" priority="9">
+    <cfRule type="expression" dxfId="91" priority="10">
       <formula>AND($M2&lt;&gt;"", $M2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="90" priority="10">
+    <cfRule type="expression" dxfId="90" priority="11">
       <formula>$M2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N17">
-    <cfRule type="expression" dxfId="89" priority="11">
+    <cfRule type="expression" dxfId="89" priority="12">
       <formula>AND($N2&lt;&gt;"", $N2&gt;=0, $N2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="88" priority="12">
+    <cfRule type="expression" dxfId="88" priority="13">
       <formula>AND($N2&lt;&gt;"", $N2&gt;5, $N2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="87" priority="13">
+    <cfRule type="expression" dxfId="87" priority="14">
       <formula>AND($N2&lt;&gt;"", $N2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="86" priority="14">
+    <cfRule type="expression" dxfId="86" priority="15">
       <formula>AND($N2&lt;&gt;"", $N2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="85" priority="15">
+    <cfRule type="expression" dxfId="85" priority="16">
       <formula>$N2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:U17">
-    <cfRule type="expression" dxfId="84" priority="16">
+    <cfRule type="expression" dxfId="84" priority="17">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="83" priority="17">
+    <cfRule type="expression" dxfId="83" priority="18">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="82" priority="18">
+    <cfRule type="expression" dxfId="82" priority="19">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="81" priority="19">
+    <cfRule type="expression" dxfId="81" priority="20">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="80" priority="20">
+    <cfRule type="expression" dxfId="80" priority="21">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:AN1000">
-    <cfRule type="expression" dxfId="100" priority="21">
+    <cfRule type="expression" dxfId="100" priority="22">
       <formula>TRIM($A2)="PAID"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="101" priority="22">
+    <cfRule type="expression" dxfId="101" priority="23">
       <formula>TRIM($A2)="Finalized"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="102" priority="23">
+    <cfRule type="expression" dxfId="102" priority="24">
       <formula>TRIM($A2)="Received"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="103" priority="24">
+    <cfRule type="expression" dxfId="103" priority="25">
       <formula>TRIM($A2)="Pending"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="104" priority="25">
+    <cfRule type="expression" dxfId="104" priority="26">
       <formula>TRIM($A2)="Under Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="105" priority="26">
+    <cfRule type="expression" dxfId="105" priority="27">
       <formula>AND(TRIM($A2)="Denied",$K2="")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="108" priority="29">
+    <cfRule type="expression" dxfId="108" priority="30">
       <formula>AND(TRIM($A2)="Denied",$K2&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="106" priority="27">
+    <cfRule type="expression" dxfId="106" priority="28">
       <formula>TRIM($A2)="Rejected"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="107" priority="28">
+    <cfRule type="expression" dxfId="107" priority="29">
       <formula>TRIM($A2)="Not found"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5746,14 +5767,15 @@
         <v>92</v>
       </c>
       <c r="M2" s="5">
-        <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($C2="","",$C2+365-TODAY()))</f>
         <v>209</v>
       </c>
       <c r="N2" s="5">
-        <f ca="1">IF($C2="","",$C2+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($C2="","",$C2+120-TODAY()))</f>
         <v>-36</v>
       </c>
       <c r="O2" s="7">
+        <f>IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",DATE(2027,1,9))</f>
         <v>46396</v>
       </c>
       <c r="P2" s="6" t="s">
@@ -5861,14 +5883,15 @@
         <v>112</v>
       </c>
       <c r="M3" s="5">
-        <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($C3="","",$C3+365-TODAY()))</f>
         <v>257</v>
       </c>
       <c r="N3" s="5">
-        <f ca="1">IF($C3="","",$C3+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($C3="","",$C3+120-TODAY()))</f>
         <v>12</v>
       </c>
       <c r="O3" s="7">
+        <f>IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",DATE(2027,1,29))</f>
         <v>46416</v>
       </c>
       <c r="P3" s="6" t="s">
@@ -5978,14 +6001,15 @@
         <v>-187</v>
       </c>
       <c r="M4" s="5">
-        <f ca="1">IF($F4="","",$F4+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($F4="","",$F4+90-TODAY()))</f>
         <v>-187</v>
       </c>
       <c r="N4" s="5">
-        <f ca="1">IF($C4="","",$C4+60-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($C4="","",$C4+60-TODAY()))</f>
         <v>-155</v>
       </c>
       <c r="O4" s="7">
+        <f>IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",DATE(2026,4,5))</f>
         <v>46117</v>
       </c>
       <c r="P4" s="6" t="s">
@@ -6097,14 +6121,15 @@
         <v>-168</v>
       </c>
       <c r="M5" s="5">
-        <f ca="1">IF($C5="","",$C5+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($C5="","",$C5+90-TODAY()))</f>
         <v>-58</v>
       </c>
       <c r="N5" s="5">
-        <f ca="1">IF($C5="","",$C5+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($C5="","",$C5+90-TODAY()))</f>
         <v>-58</v>
       </c>
       <c r="O5" s="7">
+        <f>IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",DATE(2026,4,24))</f>
         <v>46136</v>
       </c>
       <c r="P5" s="6" t="s">
@@ -6211,20 +6236,21 @@
       <c r="K6" s="4">
         <v>46261</v>
       </c>
-      <c r="L6" s="5">
+      <c t="str" r="L6" s="5">
         <f ca="1">IF($O6="","",$O6-TODAY())</f>
-        <v>92</v>
-      </c>
-      <c r="M6" s="5">
-        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
-        <v>221</v>
-      </c>
-      <c r="N6" s="5">
-        <f ca="1">IF($C6="","",$C6+120-TODAY())</f>
-        <v>-24</v>
-      </c>
-      <c r="O6" s="7">
-        <v>46396</v>
+        <v/>
+      </c>
+      <c t="str" r="M6" s="5">
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($C6="","",$C6+365-TODAY()))</f>
+        <v/>
+      </c>
+      <c t="str" r="N6" s="5">
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($C6="","",$C6+120-TODAY()))</f>
+        <v/>
+      </c>
+      <c t="str" r="O6" s="7">
+        <f>IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",DATE(2027,1,9))</f>
+        <v/>
       </c>
       <c r="P6" s="6" t="s">
         <v>46</v>
@@ -6324,20 +6350,21 @@
       <c r="K7" s="4">
         <v>46261</v>
       </c>
-      <c r="L7" s="5">
+      <c t="str" r="L7" s="5">
         <f ca="1">IF($O7="","",$O7-TODAY())</f>
-        <v>102</v>
-      </c>
-      <c r="M7" s="5">
-        <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
-        <v>147</v>
-      </c>
-      <c r="N7" s="5">
-        <f ca="1">IF($C7="","",$C7+120-TODAY())</f>
-        <v>-98</v>
-      </c>
-      <c r="O7" s="7">
-        <v>46406</v>
+        <v/>
+      </c>
+      <c t="str" r="M7" s="5">
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($C7="","",$C7+365-TODAY()))</f>
+        <v/>
+      </c>
+      <c t="str" r="N7" s="5">
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($C7="","",$C7+120-TODAY()))</f>
+        <v/>
+      </c>
+      <c t="str" r="O7" s="7">
+        <f>IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",DATE(2027,1,19))</f>
+        <v/>
       </c>
       <c r="P7" s="6" t="s">
         <v>46</v>
@@ -6439,20 +6466,21 @@
       <c r="K8" s="4">
         <v>46261</v>
       </c>
-      <c r="L8" s="5">
+      <c t="str" r="L8" s="5">
         <f ca="1">IF($O8="","",$O8-TODAY())</f>
-        <v>102</v>
-      </c>
-      <c r="M8" s="5">
-        <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
-        <v>132</v>
-      </c>
-      <c r="N8" s="5">
-        <f ca="1">IF($C8="","",$C8+120-TODAY())</f>
-        <v>-113</v>
-      </c>
-      <c r="O8" s="7">
-        <v>46406</v>
+        <v/>
+      </c>
+      <c t="str" r="M8" s="5">
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($C8="","",$C8+365-TODAY()))</f>
+        <v/>
+      </c>
+      <c t="str" r="N8" s="5">
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($C8="","",$C8+120-TODAY()))</f>
+        <v/>
+      </c>
+      <c t="str" r="O8" s="7">
+        <f>IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",DATE(2027,1,19))</f>
+        <v/>
       </c>
       <c r="P8" s="6" t="s">
         <v>46</v>
@@ -6522,100 +6550,105 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AN8" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <conditionalFormatting sqref="L2:O1000">
+    <cfRule type="expression" dxfId="101" priority="1" stopIfTrue="1">
+      <formula>AND(TRIM($A2)="Finalized",$K2&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L2:L8">
-    <cfRule type="expression" dxfId="79" priority="1">
+    <cfRule type="expression" dxfId="79" priority="2">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="78" priority="2">
+    <cfRule type="expression" dxfId="78" priority="3">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="77" priority="3">
+    <cfRule type="expression" dxfId="77" priority="4">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="76" priority="4">
+    <cfRule type="expression" dxfId="76" priority="5">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="75" priority="5">
+    <cfRule type="expression" dxfId="75" priority="6">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M8">
-    <cfRule type="expression" dxfId="74" priority="6">
+    <cfRule type="expression" dxfId="74" priority="7">
       <formula>AND($M2&lt;&gt;"", $M2&gt;=0, $M2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="7">
+    <cfRule type="expression" dxfId="73" priority="8">
       <formula>AND($M2&lt;&gt;"", $M2&gt;5, $M2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="72" priority="8">
+    <cfRule type="expression" dxfId="72" priority="9">
       <formula>AND($M2&lt;&gt;"", $M2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="71" priority="9">
+    <cfRule type="expression" dxfId="71" priority="10">
       <formula>AND($M2&lt;&gt;"", $M2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="70" priority="10">
+    <cfRule type="expression" dxfId="70" priority="11">
       <formula>$M2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N8">
-    <cfRule type="expression" dxfId="69" priority="11">
+    <cfRule type="expression" dxfId="69" priority="12">
       <formula>AND($N2&lt;&gt;"", $N2&gt;=0, $N2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="12">
+    <cfRule type="expression" dxfId="68" priority="13">
       <formula>AND($N2&lt;&gt;"", $N2&gt;5, $N2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="67" priority="13">
+    <cfRule type="expression" dxfId="67" priority="14">
       <formula>AND($N2&lt;&gt;"", $N2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="66" priority="14">
+    <cfRule type="expression" dxfId="66" priority="15">
       <formula>AND($N2&lt;&gt;"", $N2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="65" priority="15">
+    <cfRule type="expression" dxfId="65" priority="16">
       <formula>$N2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:U8">
-    <cfRule type="expression" dxfId="64" priority="16">
+    <cfRule type="expression" dxfId="64" priority="17">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="17">
+    <cfRule type="expression" dxfId="63" priority="18">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="62" priority="18">
+    <cfRule type="expression" dxfId="62" priority="19">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="61" priority="19">
+    <cfRule type="expression" dxfId="61" priority="20">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="20">
+    <cfRule type="expression" dxfId="60" priority="21">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:AN1000">
-    <cfRule type="expression" dxfId="100" priority="21">
+    <cfRule type="expression" dxfId="100" priority="22">
       <formula>TRIM($A2)="PAID"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="101" priority="22">
+    <cfRule type="expression" dxfId="101" priority="23">
       <formula>TRIM($A2)="Finalized"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="102" priority="23">
+    <cfRule type="expression" dxfId="102" priority="24">
       <formula>TRIM($A2)="Received"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="103" priority="24">
+    <cfRule type="expression" dxfId="103" priority="25">
       <formula>TRIM($A2)="Pending"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="104" priority="25">
+    <cfRule type="expression" dxfId="104" priority="26">
       <formula>TRIM($A2)="Under Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="105" priority="26">
+    <cfRule type="expression" dxfId="105" priority="27">
       <formula>AND(TRIM($A2)="Denied",$K2="")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="108" priority="29">
+    <cfRule type="expression" dxfId="108" priority="30">
       <formula>AND(TRIM($A2)="Denied",$K2&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="106" priority="27">
+    <cfRule type="expression" dxfId="106" priority="28">
       <formula>TRIM($A2)="Rejected"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="107" priority="28">
+    <cfRule type="expression" dxfId="107" priority="29">
       <formula>TRIM($A2)="Not found"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6828,14 +6861,15 @@
         <v>95</v>
       </c>
       <c r="M2" s="5">
-        <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($C2="","",$C2+365-TODAY()))</f>
         <v>196</v>
       </c>
       <c r="N2" s="5">
-        <f ca="1">IF($C2="","",$C2+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($C2="","",$C2+120-TODAY()))</f>
         <v>-49</v>
       </c>
       <c r="O2" s="7">
+        <f>IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",DATE(2027,1,12))</f>
         <v>46399</v>
       </c>
       <c r="P2" s="6" t="s">
@@ -6945,14 +6979,15 @@
         <v>102</v>
       </c>
       <c r="M3" s="5">
-        <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($C3="","",$C3+365-TODAY()))</f>
         <v>208</v>
       </c>
       <c r="N3" s="5">
-        <f ca="1">IF($C3="","",$C3+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($C3="","",$C3+120-TODAY()))</f>
         <v>-37</v>
       </c>
       <c r="O3" s="7">
+        <f>IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",DATE(2027,1,19))</f>
         <v>46406</v>
       </c>
       <c r="P3" s="6" t="s">
@@ -7058,14 +7093,15 @@
         <v>102</v>
       </c>
       <c r="M4" s="5">
-        <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($C4="","",$C4+365-TODAY()))</f>
         <v>196</v>
       </c>
       <c r="N4" s="5">
-        <f ca="1">IF($C4="","",$C4+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($C4="","",$C4+120-TODAY()))</f>
         <v>-49</v>
       </c>
       <c r="O4" s="7">
+        <f>IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",DATE(2027,1,19))</f>
         <v>46406</v>
       </c>
       <c r="P4" s="6" t="s">
@@ -7177,14 +7213,15 @@
         <v>102</v>
       </c>
       <c r="M5" s="5">
-        <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($C5="","",$C5+365-TODAY()))</f>
         <v>181</v>
       </c>
       <c r="N5" s="5">
-        <f ca="1">IF($C5="","",$C5+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($C5="","",$C5+120-TODAY()))</f>
         <v>-64</v>
       </c>
       <c r="O5" s="7">
+        <f>IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",DATE(2027,1,19))</f>
         <v>46406</v>
       </c>
       <c r="P5" s="6" t="s">
@@ -7296,14 +7333,15 @@
         <v>109</v>
       </c>
       <c r="M6" s="5">
-        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($C6="","",$C6+365-TODAY()))</f>
         <v>181</v>
       </c>
       <c r="N6" s="5">
-        <f ca="1">IF($C6="","",$C6+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($C6="","",$C6+120-TODAY()))</f>
         <v>-64</v>
       </c>
       <c r="O6" s="7">
+        <f>IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",DATE(2027,1,26))</f>
         <v>46413</v>
       </c>
       <c r="P6" s="6" t="s">
@@ -7415,14 +7453,15 @@
         <v>109</v>
       </c>
       <c r="M7" s="5">
-        <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($C7="","",$C7+365-TODAY()))</f>
         <v>160</v>
       </c>
       <c r="N7" s="5">
-        <f ca="1">IF($C7="","",$C7+120-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($C7="","",$C7+120-TODAY()))</f>
         <v>-85</v>
       </c>
       <c r="O7" s="7">
+        <f>IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",DATE(2027,1,26))</f>
         <v>46413</v>
       </c>
       <c r="P7" s="6" t="s">
@@ -7530,14 +7569,15 @@
         <v>-187</v>
       </c>
       <c r="M8" s="5">
-        <f ca="1">IF($F8="","",$F8+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($F8="","",$F8+90-TODAY()))</f>
         <v>-187</v>
       </c>
       <c r="N8" s="5">
-        <f ca="1">IF($C8="","",$C8+540-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($C8="","",$C8+540-TODAY()))</f>
         <v>357</v>
       </c>
       <c r="O8" s="7">
+        <f>IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",DATE(2026,4,5))</f>
         <v>46117</v>
       </c>
       <c r="P8" s="6" t="s">
@@ -7643,14 +7683,15 @@
         <v>-187</v>
       </c>
       <c r="M9" s="5">
-        <f ca="1">IF($F9="","",$F9+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A9)="Finalized",$K9&lt;&gt;""),"",IF($F9="","",$F9+90-TODAY()))</f>
         <v>-187</v>
       </c>
       <c r="N9" s="5">
-        <f ca="1">IF($C9="","",$C9+540-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A9)="Finalized",$K9&lt;&gt;""),"",IF($C9="","",$C9+540-TODAY()))</f>
         <v>378</v>
       </c>
       <c r="O9" s="7">
+        <f>IF(AND(TRIM($A9)="Finalized",$K9&lt;&gt;""),"",DATE(2026,4,5))</f>
         <v>46117</v>
       </c>
       <c r="P9" s="6" t="s">
@@ -7756,14 +7797,15 @@
         <v>-166</v>
       </c>
       <c r="M10" s="5">
-        <f ca="1">IF($F10="","",$F10+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A10)="Finalized",$K10&lt;&gt;""),"",IF($F10="","",$F10+90-TODAY()))</f>
         <v>-166</v>
       </c>
       <c r="N10" s="5">
-        <f ca="1">IF($C10="","",$C10+540-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A10)="Finalized",$K10&lt;&gt;""),"",IF($C10="","",$C10+540-TODAY()))</f>
         <v>347</v>
       </c>
       <c r="O10" s="7">
+        <f>IF(AND(TRIM($A10)="Finalized",$K10&lt;&gt;""),"",DATE(2026,4,26))</f>
         <v>46138</v>
       </c>
       <c r="P10" s="6" t="s">
@@ -7869,14 +7911,15 @@
         <v>-157</v>
       </c>
       <c r="M11" s="5">
-        <f ca="1">IF($C11="","",$C11+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A11)="Finalized",$K11&lt;&gt;""),"",IF($C11="","",$C11+180-TODAY()))</f>
         <v>3</v>
       </c>
       <c r="N11" s="5">
-        <f ca="1">IF($C11="","",$C11+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A11)="Finalized",$K11&lt;&gt;""),"",IF($C11="","",$C11+180-TODAY()))</f>
         <v>3</v>
       </c>
       <c r="O11" s="7">
+        <f>IF(AND(TRIM($A11)="Finalized",$K11&lt;&gt;""),"",DATE(2026,5,5))</f>
         <v>46147</v>
       </c>
       <c r="P11" s="6" t="s">
@@ -7983,7 +8026,7 @@
       </c>
       <c r="M12" s="5"/>
       <c r="N12" s="5">
-        <f ca="1">IF($C12="","",$C12+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A12)="Finalized",$K12&lt;&gt;""),"",IF($C12="","",$C12+180-TODAY()))</f>
         <v>17</v>
       </c>
       <c r="O12" s="7"/>
@@ -8053,100 +8096,105 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AN12" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="L2:O1000">
+    <cfRule type="expression" dxfId="101" priority="1" stopIfTrue="1">
+      <formula>AND(TRIM($A2)="Finalized",$K2&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L2:L12">
-    <cfRule type="expression" dxfId="59" priority="1">
+    <cfRule type="expression" dxfId="59" priority="2">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="58" priority="2">
+    <cfRule type="expression" dxfId="58" priority="3">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="57" priority="3">
+    <cfRule type="expression" dxfId="57" priority="4">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="56" priority="4">
+    <cfRule type="expression" dxfId="56" priority="5">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="5">
+    <cfRule type="expression" dxfId="55" priority="6">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M12">
-    <cfRule type="expression" dxfId="54" priority="6">
+    <cfRule type="expression" dxfId="54" priority="7">
       <formula>AND($M2&lt;&gt;"", $M2&gt;=0, $M2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="53" priority="7">
+    <cfRule type="expression" dxfId="53" priority="8">
       <formula>AND($M2&lt;&gt;"", $M2&gt;5, $M2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="52" priority="8">
+    <cfRule type="expression" dxfId="52" priority="9">
       <formula>AND($M2&lt;&gt;"", $M2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="9">
+    <cfRule type="expression" dxfId="51" priority="10">
       <formula>AND($M2&lt;&gt;"", $M2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="50" priority="10">
+    <cfRule type="expression" dxfId="50" priority="11">
       <formula>$M2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N12">
-    <cfRule type="expression" dxfId="49" priority="11">
+    <cfRule type="expression" dxfId="49" priority="12">
       <formula>AND($N2&lt;&gt;"", $N2&gt;=0, $N2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="12">
+    <cfRule type="expression" dxfId="48" priority="13">
       <formula>AND($N2&lt;&gt;"", $N2&gt;5, $N2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="47" priority="13">
+    <cfRule type="expression" dxfId="47" priority="14">
       <formula>AND($N2&lt;&gt;"", $N2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="46" priority="14">
+    <cfRule type="expression" dxfId="46" priority="15">
       <formula>AND($N2&lt;&gt;"", $N2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="15">
+    <cfRule type="expression" dxfId="45" priority="16">
       <formula>$N2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:U12">
-    <cfRule type="expression" dxfId="44" priority="16">
+    <cfRule type="expression" dxfId="44" priority="17">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="43" priority="17">
+    <cfRule type="expression" dxfId="43" priority="18">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="18">
+    <cfRule type="expression" dxfId="42" priority="19">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="19">
+    <cfRule type="expression" dxfId="41" priority="20">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="20">
+    <cfRule type="expression" dxfId="40" priority="21">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:AN1000">
-    <cfRule type="expression" dxfId="100" priority="21">
+    <cfRule type="expression" dxfId="100" priority="22">
       <formula>TRIM($A2)="PAID"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="101" priority="22">
+    <cfRule type="expression" dxfId="101" priority="23">
       <formula>TRIM($A2)="Finalized"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="102" priority="23">
+    <cfRule type="expression" dxfId="102" priority="24">
       <formula>TRIM($A2)="Received"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="103" priority="24">
+    <cfRule type="expression" dxfId="103" priority="25">
       <formula>TRIM($A2)="Pending"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="104" priority="25">
+    <cfRule type="expression" dxfId="104" priority="26">
       <formula>TRIM($A2)="Under Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="105" priority="26">
+    <cfRule type="expression" dxfId="105" priority="27">
       <formula>AND(TRIM($A2)="Denied",$K2="")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="108" priority="29">
+    <cfRule type="expression" dxfId="108" priority="30">
       <formula>AND(TRIM($A2)="Denied",$K2&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="106" priority="27">
+    <cfRule type="expression" dxfId="106" priority="28">
       <formula>TRIM($A2)="Rejected"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="107" priority="28">
+    <cfRule type="expression" dxfId="107" priority="29">
       <formula>TRIM($A2)="Not found"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8355,14 +8403,15 @@
         <v>-207</v>
       </c>
       <c r="M2" s="5" t="str">
-        <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($C2="","",$C2+365-TODAY()))</f>
         <v/>
       </c>
       <c r="N2" s="5" t="str">
-        <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($C2="","",$C2+365-TODAY()))</f>
         <v/>
       </c>
       <c r="O2" s="7">
+        <f>IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",DATE(2026,3,16))</f>
         <v>46097</v>
       </c>
       <c r="P2" s="6" t="s">
@@ -8462,14 +8511,15 @@
         <v>-183</v>
       </c>
       <c r="M3" s="5">
-        <f ca="1">IF($F3="","",$F3+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($F3="","",$F3+90-TODAY()))</f>
         <v>-183</v>
       </c>
       <c r="N3" s="5">
-        <f ca="1">IF($C3="","",$C3+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($C3="","",$C3+180-TODAY()))</f>
         <v>-12</v>
       </c>
       <c r="O3" s="7">
+        <f>IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",DATE(2026,4,9))</f>
         <v>46121</v>
       </c>
       <c r="P3" s="6" t="s">
@@ -8569,14 +8619,15 @@
         <v>-183</v>
       </c>
       <c r="M4" s="5">
-        <f ca="1">IF($C4="","",$C4+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($C4="","",$C4+180-TODAY()))</f>
         <v>32</v>
       </c>
       <c r="N4" s="5">
-        <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($C4="","",$C4+365-TODAY()))</f>
         <v>217</v>
       </c>
       <c r="O4" s="7">
+        <f>IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",DATE(2026,4,9))</f>
         <v>46121</v>
       </c>
       <c r="P4" s="6" t="s">
@@ -8676,14 +8727,15 @@
         <v>-179</v>
       </c>
       <c r="M5" s="5">
-        <f ca="1">IF($C5="","",$C5+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($C5="","",$C5+180-TODAY()))</f>
         <v>-79</v>
       </c>
       <c r="N5" s="5">
-        <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($C5="","",$C5+365-TODAY()))</f>
         <v>106</v>
       </c>
       <c r="O5" s="7">
+        <f>IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",DATE(2026,4,13))</f>
         <v>46125</v>
       </c>
       <c r="P5" s="6" t="s">
@@ -8781,14 +8833,15 @@
         <v>-178</v>
       </c>
       <c r="M6" s="5">
-        <f ca="1">IF($F6="","",$F6+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($F6="","",$F6+90-TODAY()))</f>
         <v>-178</v>
       </c>
       <c r="N6" s="5" t="str">
-        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($C6="","",$C6+365-TODAY()))</f>
         <v/>
       </c>
       <c r="O6" s="7">
+        <f>IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",DATE(2026,4,14))</f>
         <v>46126</v>
       </c>
       <c r="P6" s="6" t="s">
@@ -8888,14 +8941,15 @@
         <v>-169</v>
       </c>
       <c r="M7" s="5">
-        <f ca="1">IF($F7="","",$F7+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($F7="","",$F7+90-TODAY()))</f>
         <v>-169</v>
       </c>
       <c r="N7" s="5">
-        <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($C7="","",$C7+365-TODAY()))</f>
         <v>224</v>
       </c>
       <c r="O7" s="7">
+        <f>IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",DATE(2026,4,23))</f>
         <v>46135</v>
       </c>
       <c r="P7" s="6" t="s">
@@ -9001,14 +9055,15 @@
         <v>-169</v>
       </c>
       <c r="M8" s="5">
-        <f ca="1">IF($F8="","",$F8+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($F8="","",$F8+90-TODAY()))</f>
         <v>-169</v>
       </c>
       <c r="N8" s="5">
-        <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($C8="","",$C8+365-TODAY()))</f>
         <v>113</v>
       </c>
       <c r="O8" s="7">
+        <f>IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",DATE(2026,4,23))</f>
         <v>46135</v>
       </c>
       <c r="P8" s="6" t="s">
@@ -9261,100 +9316,105 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AN10" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="L2:O1000">
+    <cfRule type="expression" dxfId="101" priority="1" stopIfTrue="1">
+      <formula>AND(TRIM($A2)="Finalized",$K2&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L2:L10">
-    <cfRule type="expression" dxfId="39" priority="1">
+    <cfRule type="expression" dxfId="39" priority="2">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="2">
+    <cfRule type="expression" dxfId="38" priority="3">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="3">
+    <cfRule type="expression" dxfId="37" priority="4">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="4">
+    <cfRule type="expression" dxfId="36" priority="5">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="5">
+    <cfRule type="expression" dxfId="35" priority="6">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M10">
-    <cfRule type="expression" dxfId="34" priority="6">
+    <cfRule type="expression" dxfId="34" priority="7">
       <formula>AND($M2&lt;&gt;"", $M2&gt;=0, $M2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="7">
+    <cfRule type="expression" dxfId="33" priority="8">
       <formula>AND($M2&lt;&gt;"", $M2&gt;5, $M2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="8">
+    <cfRule type="expression" dxfId="32" priority="9">
       <formula>AND($M2&lt;&gt;"", $M2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="9">
+    <cfRule type="expression" dxfId="31" priority="10">
       <formula>AND($M2&lt;&gt;"", $M2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="10">
+    <cfRule type="expression" dxfId="30" priority="11">
       <formula>$M2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N10">
-    <cfRule type="expression" dxfId="29" priority="11">
+    <cfRule type="expression" dxfId="29" priority="12">
       <formula>AND($N2&lt;&gt;"", $N2&gt;=0, $N2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="12">
+    <cfRule type="expression" dxfId="28" priority="13">
       <formula>AND($N2&lt;&gt;"", $N2&gt;5, $N2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="13">
+    <cfRule type="expression" dxfId="27" priority="14">
       <formula>AND($N2&lt;&gt;"", $N2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="14">
+    <cfRule type="expression" dxfId="26" priority="15">
       <formula>AND($N2&lt;&gt;"", $N2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="15">
+    <cfRule type="expression" dxfId="25" priority="16">
       <formula>$N2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:U10">
-    <cfRule type="expression" dxfId="24" priority="16">
+    <cfRule type="expression" dxfId="24" priority="17">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="17">
+    <cfRule type="expression" dxfId="23" priority="18">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="18">
+    <cfRule type="expression" dxfId="22" priority="19">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="19">
+    <cfRule type="expression" dxfId="21" priority="20">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="20">
+    <cfRule type="expression" dxfId="20" priority="21">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:AN1000">
-    <cfRule type="expression" dxfId="100" priority="21">
+    <cfRule type="expression" dxfId="100" priority="22">
       <formula>TRIM($A2)="PAID"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="101" priority="22">
+    <cfRule type="expression" dxfId="101" priority="23">
       <formula>TRIM($A2)="Finalized"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="102" priority="23">
+    <cfRule type="expression" dxfId="102" priority="24">
       <formula>TRIM($A2)="Received"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="103" priority="24">
+    <cfRule type="expression" dxfId="103" priority="25">
       <formula>TRIM($A2)="Pending"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="104" priority="25">
+    <cfRule type="expression" dxfId="104" priority="26">
       <formula>TRIM($A2)="Under Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="105" priority="26">
+    <cfRule type="expression" dxfId="105" priority="27">
       <formula>AND(TRIM($A2)="Denied",$K2="")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="108" priority="29">
+    <cfRule type="expression" dxfId="108" priority="30">
       <formula>AND(TRIM($A2)="Denied",$K2&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="106" priority="27">
+    <cfRule type="expression" dxfId="106" priority="28">
       <formula>TRIM($A2)="Rejected"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="107" priority="28">
+    <cfRule type="expression" dxfId="107" priority="29">
       <formula>TRIM($A2)="Not found"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9567,14 +9627,15 @@
         <v>-184</v>
       </c>
       <c r="M2" s="5">
-        <f ca="1">IF($F2="","",$F2+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($F2="","",$F2+90-TODAY()))</f>
         <v>-184</v>
       </c>
       <c r="N2" s="5">
-        <f ca="1">IF($C2="","",$C2+540-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",IF($C2="","",$C2+540-TODAY()))</f>
         <v>435</v>
       </c>
       <c r="O2" s="7">
+        <f>IF(AND(TRIM($A2)="Finalized",$K2&lt;&gt;""),"",DATE(2026,4,8))</f>
         <v>46120</v>
       </c>
       <c r="P2" s="6" t="s">
@@ -9670,14 +9731,15 @@
         <v>-184</v>
       </c>
       <c r="M3" s="5" t="str">
-        <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($C3="","",$C3+365-TODAY()))</f>
         <v/>
       </c>
       <c r="N3" s="5" t="str">
-        <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",IF($C3="","",$C3+365-TODAY()))</f>
         <v/>
       </c>
       <c r="O3" s="7">
+        <f>IF(AND(TRIM($A3)="Finalized",$K3&lt;&gt;""),"",DATE(2026,4,8))</f>
         <v>46120</v>
       </c>
       <c r="P3" s="6" t="s">
@@ -9779,14 +9841,15 @@
         <v>-179</v>
       </c>
       <c r="M4" s="5">
-        <f ca="1">IF($F4="","",$F4+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($F4="","",$F4+90-TODAY()))</f>
         <v>-179</v>
       </c>
       <c r="N4" s="5">
-        <f ca="1">IF($C4="","",$C4+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",IF($C4="","",$C4+180-TODAY()))</f>
         <v>-55</v>
       </c>
       <c r="O4" s="7">
+        <f>IF(AND(TRIM($A4)="Finalized",$K4&lt;&gt;""),"",DATE(2026,4,13))</f>
         <v>46125</v>
       </c>
       <c r="P4" s="6" t="s">
@@ -9886,14 +9949,15 @@
         <v>-178</v>
       </c>
       <c r="M5" s="5">
-        <f ca="1">IF($F5="","",$F5+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($F5="","",$F5+90-TODAY()))</f>
         <v>-178</v>
       </c>
       <c r="N5" s="5">
-        <f ca="1">IF($C5="","",$C5+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",IF($C5="","",$C5+180-TODAY()))</f>
         <v>36</v>
       </c>
       <c r="O5" s="7">
+        <f>IF(AND(TRIM($A5)="Finalized",$K5&lt;&gt;""),"",DATE(2026,4,14))</f>
         <v>46126</v>
       </c>
       <c r="P5" s="6" t="s">
@@ -9997,14 +10061,15 @@
         <v>-177</v>
       </c>
       <c r="M6" s="5">
-        <f ca="1">IF($C6="","",$C6+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($C6="","",$C6+180-TODAY()))</f>
         <v>39</v>
       </c>
       <c r="N6" s="5">
-        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",IF($C6="","",$C6+365-TODAY()))</f>
         <v>224</v>
       </c>
       <c r="O6" s="7">
+        <f>IF(AND(TRIM($A6)="Finalized",$K6&lt;&gt;""),"",DATE(2026,4,15))</f>
         <v>46127</v>
       </c>
       <c r="P6" s="6" t="s">
@@ -10106,14 +10171,15 @@
         <v>-171</v>
       </c>
       <c r="M7" s="5">
-        <f ca="1">IF($F7="","",$F7+90-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($F7="","",$F7+90-TODAY()))</f>
         <v>-171</v>
       </c>
       <c r="N7" s="5">
-        <f ca="1">IF($C7="","",$C7+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",IF($C7="","",$C7+180-TODAY()))</f>
         <v>36</v>
       </c>
       <c r="O7" s="7">
+        <f>IF(AND(TRIM($A7)="Finalized",$K7&lt;&gt;""),"",DATE(2026,4,21))</f>
         <v>46133</v>
       </c>
       <c r="P7" s="6" t="s">
@@ -10213,14 +10279,15 @@
         <v>-163</v>
       </c>
       <c r="M8" s="5">
-        <f ca="1">IF($C8="","",$C8+180-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($C8="","",$C8+180-TODAY()))</f>
         <v>32</v>
       </c>
       <c r="N8" s="5">
-        <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
+        <f ca="1">IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",IF($C8="","",$C8+365-TODAY()))</f>
         <v>217</v>
       </c>
       <c r="O8" s="7">
+        <f>IF(AND(TRIM($A8)="Finalized",$K8&lt;&gt;""),"",DATE(2026,4,29))</f>
         <v>46141</v>
       </c>
       <c r="P8" s="6" t="s">
@@ -10291,100 +10358,105 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AN8" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <conditionalFormatting sqref="L2:O1000">
+    <cfRule type="expression" dxfId="101" priority="1" stopIfTrue="1">
+      <formula>AND(TRIM($A2)="Finalized",$K2&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L2:L8">
-    <cfRule type="expression" dxfId="19" priority="1">
+    <cfRule type="expression" dxfId="19" priority="2">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="3">
+    <cfRule type="expression" dxfId="17" priority="4">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="4">
+    <cfRule type="expression" dxfId="16" priority="5">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="5">
+    <cfRule type="expression" dxfId="15" priority="6">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M8">
-    <cfRule type="expression" dxfId="14" priority="6">
+    <cfRule type="expression" dxfId="14" priority="7">
       <formula>AND($M2&lt;&gt;"", $M2&gt;=0, $M2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="7">
+    <cfRule type="expression" dxfId="13" priority="8">
       <formula>AND($M2&lt;&gt;"", $M2&gt;5, $M2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="8">
+    <cfRule type="expression" dxfId="12" priority="9">
       <formula>AND($M2&lt;&gt;"", $M2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="9">
+    <cfRule type="expression" dxfId="11" priority="10">
       <formula>AND($M2&lt;&gt;"", $M2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="10">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>$M2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N8">
-    <cfRule type="expression" dxfId="9" priority="11">
+    <cfRule type="expression" dxfId="9" priority="12">
       <formula>AND($N2&lt;&gt;"", $N2&gt;=0, $N2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="12">
+    <cfRule type="expression" dxfId="8" priority="13">
       <formula>AND($N2&lt;&gt;"", $N2&gt;5, $N2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="13">
+    <cfRule type="expression" dxfId="7" priority="14">
       <formula>AND($N2&lt;&gt;"", $N2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="14">
+    <cfRule type="expression" dxfId="6" priority="15">
       <formula>AND($N2&lt;&gt;"", $N2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="15">
+    <cfRule type="expression" dxfId="5" priority="16">
       <formula>$N2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:U8">
-    <cfRule type="expression" dxfId="4" priority="16">
+    <cfRule type="expression" dxfId="4" priority="17">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="17">
+    <cfRule type="expression" dxfId="3" priority="18">
       <formula>AND($L2&lt;&gt;"", $L2&gt;5, $L2&lt;=30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="18">
+    <cfRule type="expression" dxfId="2" priority="19">
       <formula>AND($L2&lt;&gt;"", $L2&gt;30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="19">
+    <cfRule type="expression" dxfId="1" priority="20">
       <formula>AND($L2&lt;&gt;"", $L2&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="20">
+    <cfRule type="expression" dxfId="0" priority="21">
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:AN1000">
-    <cfRule type="expression" dxfId="100" priority="21">
+    <cfRule type="expression" dxfId="100" priority="22">
       <formula>TRIM($A2)="PAID"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="101" priority="22">
+    <cfRule type="expression" dxfId="101" priority="23">
       <formula>TRIM($A2)="Finalized"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="102" priority="23">
+    <cfRule type="expression" dxfId="102" priority="24">
       <formula>TRIM($A2)="Received"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="103" priority="24">
+    <cfRule type="expression" dxfId="103" priority="25">
       <formula>TRIM($A2)="Pending"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="104" priority="25">
+    <cfRule type="expression" dxfId="104" priority="26">
       <formula>TRIM($A2)="Under Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="105" priority="26">
+    <cfRule type="expression" dxfId="105" priority="27">
       <formula>AND(TRIM($A2)="Denied",$K2="")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="108" priority="29">
+    <cfRule type="expression" dxfId="108" priority="30">
       <formula>AND(TRIM($A2)="Denied",$K2&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="106" priority="27">
+    <cfRule type="expression" dxfId="106" priority="28">
       <formula>TRIM($A2)="Rejected"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="107" priority="28">
+    <cfRule type="expression" dxfId="107" priority="29">
       <formula>TRIM($A2)="Not found"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10456,7 +10528,7 @@
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="str">
         <f>"    3 - Due in 31+ days: "&amp;SUM(COUNTIFS(BH!$L$2:$L$1000,"&gt;30"),COUNTIFS(DME!$L$2:$L$1000,"&gt;30"),COUNTIFS(GAE!$L$2:$L$1000,"&gt;30"),COUNTIFS(ORTHO!$L$2:$L$1000,"&gt;30"),COUNTIFS(US!$L$2:$L$1000,"&gt;30"))</f>
-        <v>    3 - Due in 31+ days: 15</v>
+        <v>    3 - Due in 31+ days: 12</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -10467,7 +10539,7 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="str">
-        <f>"    5 - No limit on file: "&amp;SUM(COUNTIFS(BH!$D$2:$D$1000,"&lt;&gt;",BH!$L$2:$L$1000,""),COUNTIFS(DME!$D$2:$D$1000,"&lt;&gt;",DME!$L$2:$L$1000,""),COUNTIFS(GAE!$D$2:$D$1000,"&lt;&gt;",GAE!$L$2:$L$1000,""),COUNTIFS(ORTHO!$D$2:$D$1000,"&lt;&gt;",ORTHO!$L$2:$L$1000,""),COUNTIFS(US!$D$2:$D$1000,"&lt;&gt;",US!$L$2:$L$1000,""))</f>
+        <f>"    5 - No limit on file: "&amp;SUM(SUMPRODUCT((BH!$D$2:$D$1000&lt;&gt;"")*(BH!$L$2:$L$1000="")*(1-(TRIM(BH!$A$2:$A$1000)="Finalized")*(BH!$K$2:$K$1000&lt;&gt;""))),SUMPRODUCT((DME!$D$2:$D$1000&lt;&gt;"")*(DME!$L$2:$L$1000="")*(1-(TRIM(DME!$A$2:$A$1000)="Finalized")*(DME!$K$2:$K$1000&lt;&gt;""))),SUMPRODUCT((GAE!$D$2:$D$1000&lt;&gt;"")*(GAE!$L$2:$L$1000="")*(1-(TRIM(GAE!$A$2:$A$1000)="Finalized")*(GAE!$K$2:$K$1000&lt;&gt;""))),SUMPRODUCT((ORTHO!$D$2:$D$1000&lt;&gt;"")*(ORTHO!$L$2:$L$1000="")*(1-(TRIM(ORTHO!$A$2:$A$1000)="Finalized")*(ORTHO!$K$2:$K$1000&lt;&gt;""))),SUMPRODUCT((US!$D$2:$D$1000&lt;&gt;"")*(US!$L$2:$L$1000="")*(1-(TRIM(US!$A$2:$A$1000)="Finalized")*(US!$K$2:$K$1000&lt;&gt;""))))</f>
         <v>    5 - No limit on file: 3</v>
       </c>
     </row>

</xml_diff>